<commit_message>
Record v8 telemetry implementation in DAPHNE intake
</commit_message>
<xml_diff>
--- a/interface-data/daphne/DAPHNE_DCS_Full_Variable_Intake.xlsx
+++ b/interface-data/daphne/DAPHNE_DCS_Full_Variable_Intake.xlsx
@@ -723,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C44"/>
+  <dimension ref="B1:C44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -847,7 +847,7 @@
       </c>
       <c r="C10" s="17" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
       </c>
       <c r="C11" s="17" t="inlineStr">
         <is>
-          <t>Draft 0.7 for joint PDS / Slow Controls / DAQ / DPS review</t>
+          <t>Draft 0.8 for joint PDS / Slow Controls / DAQ / DPS review</t>
         </is>
       </c>
     </row>
@@ -2527,17 +2527,17 @@
       </c>
       <c r="B2" s="19" t="inlineStr">
         <is>
-          <t>b18075ed3e7d</t>
+          <t>feature/slow-control-emulator 8f0bbe8 (2026-08-18)</t>
         </is>
       </c>
       <c r="C2" s="19" t="inlineStr">
         <is>
-          <t>srcs/protobuf/daphneV3_*; FpgaRegDict.cpp; defines.hpp; monitoring/handlers; HD-mezz docs</t>
+          <t>daphne_v8_telemetry.proto; v8 snapshot builder/service/runtime/hardware collectors; emulator; branch audit</t>
         </is>
       </c>
       <c r="D2" s="19" t="inlineStr">
         <is>
-          <t>Current C++ control/monitor and register surface; working tree has unrelated emulator changes</t>
+          <t>Proposed-v8 typed telemetry producer and ControlEnvelopeV2/ZMQ handler; 1,370 board-owned points; feature/read_dead_time is explicitly deprecated</t>
         </is>
       </c>
     </row>
@@ -2571,17 +2571,17 @@
       </c>
       <c r="B4" s="19" t="inlineStr">
         <is>
-          <t>a3df24e0e318 + shared-gateway working tree</t>
+          <t>marroyav/rpu-afe-control d278d39 (2026-08-18)</t>
         </is>
       </c>
       <c r="C4" s="19" t="inlineStr">
         <is>
-          <t>daphne_sc.proto; Rust status collector/preflight/RPU; OPC-UA bridge</t>
+          <t>OPC-UA bridge DaphneClient; v8 validation; typed snapshot writer; registry contract and end-to-end smoke</t>
         </is>
       </c>
       <c r="D4" s="19" t="inlineStr">
         <is>
-          <t>Current NP04 bridge is a read-only proof of concept; this revision adds workbook-driven roles and mapped configuration methods</t>
+          <t>Proposed-v8 bridge maps the validated 1002/1003 snapshot into typed OPC-UA DataValues; legacy readback remains isolated as a compatibility fallback</t>
         </is>
       </c>
     </row>
@@ -2603,7 +2603,7 @@
       </c>
       <c r="D5" s="19" t="inlineStr">
         <is>
-          <t>Firmware, services, identity, network, and gateware requirements. The spy-trigger selector/inhibit at 0x88000034 is a working-tree interface not yet exposed by Protobuf/ZMQ.</t>
+          <t>Firmware, services, identity, network, and gateware requirements. The spy-trigger selector/inhibit at 0x88000034 is exposed as typed proposed-v8 Protobuf/ZMQ readback; the older spy-buffer dead-time branch is deprecated.</t>
         </is>
       </c>
     </row>

</xml_diff>